<commit_message>
Deploy TWHA IG static website (rebuild: RFP naming, Core/Extended reframing, LDL-C preferred code fix, 附表十 module audit + LOINC corrections)
</commit_message>
<xml_diff>
--- a/CodeSystem-CS-HazardType.xlsx
+++ b/CodeSystem-CS-HazardType.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-09T21:42:02+08:00</t>
+    <t>2026-07-10T19:56:53+08:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -222,7 +222,7 @@
     <t>特定化學物質作業</t>
   </si>
   <si>
-    <t>從事特定化學物質危害預防標準所定義之特定化學物質作業。</t>
+    <t>從事特定化學物質危害預防標準所定義之特定化學物質作業，涵蓋苯、氯乙烯單體、石綿、鉻、鎘、鈹、砷、汞、錳、聯苯胺類等物質作業；細分類對應請見 VS-SpecificChemicalType（呼應文件一之 18 類特定化學物質展開）。</t>
   </si>
   <si>
     <t>yellow-phosphorus</t>

</xml_diff>

<commit_message>
Deploy TWHA IG (115.06.26 sync): 附表十35項+ConceptMap, 急診摘要UC-007, RBC/MCV, performer MS
對應原始碼 commit a4b9488。本次 IG Publisher 建置產物(0 broken links)。

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CodeSystem-CS-HazardType.xlsx
+++ b/CodeSystem-CS-HazardType.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-10T21:30:50+08:00</t>
+    <t>2026-07-23T22:22:27+08:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -87,7 +87,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>勞工健康保護規則所定義之 12 大類特別危害健康作業類別。</t>
+    <t>勞工健康保護規則所定義之特別危害健康作業，歸併為 12 危害家族（家族層）。附表十（115.06.26 修正）逐號列舉之 35 項法定具名作業另以 CS-Appendix10Operation 表示，家族 ↔ 具名作業之對映見 ConceptMap Appendix10-to-HazardType。</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>